<commit_message>
Add Emma's friends as their own guest group
Twenty-five names go in as Emma / Friends, keeping the earlier batch as
Holliday / Friends (Tier 4), so the Side column separates the two lists and
each filters on its own. Totals move to 179 parties and 199 guests, and the
Overview picks up a row for the new group.

Flags three possible overlaps with names already on the sheet rather than
merging them: Jackie and Chris Santander against the parents' friends on rows
91 and 101-102, and the second Garrett against Garrett Thurmond.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rw2r7NxWEm5H3kNec61RK1
</commit_message>
<xml_diff>
--- a/guests/Wedding_Planning_Workbook.xlsx
+++ b/guests/Wedding_Planning_Workbook.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Seating Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Guest List'!$A$3:$R$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Guest List'!$A$3:$R$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B11" s="13">
-        <f>COUNTA('Guest List'!B4:B157)</f>
+        <f>COUNTA('Guest List'!B4:B182)</f>
         <v/>
       </c>
     </row>
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="B12" s="9">
-        <f>SUM('Guest List'!F4:F157)</f>
+        <f>SUM('Guest List'!F4:F182)</f>
         <v/>
       </c>
     </row>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="B13" s="13">
-        <f>COUNTIF('Guest List'!M4:M157,"Yes")</f>
+        <f>COUNTIF('Guest List'!M4:M182,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B14" s="9">
-        <f>COUNTIF('Guest List'!M4:M157,"No")</f>
+        <f>COUNTIF('Guest List'!M4:M182,"No")</f>
         <v/>
       </c>
     </row>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="B15" s="13">
-        <f>COUNTIF('Guest List'!M4:M157,"Pending")</f>
+        <f>COUNTIF('Guest List'!M4:M182,"Pending")</f>
         <v/>
       </c>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B16" s="9">
-        <f>SUM('Guest List'!N4:N157)</f>
+        <f>SUM('Guest List'!N4:N182)</f>
         <v/>
       </c>
     </row>
@@ -773,11 +773,11 @@
         </is>
       </c>
       <c r="C20" s="15">
-        <f>COUNTIFS('Guest List'!C4:C157,A20,'Guest List'!D4:D157,B20)</f>
+        <f>COUNTIFS('Guest List'!C4:C182,A20,'Guest List'!D4:D182,B20)</f>
         <v/>
       </c>
       <c r="D20" s="15">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A20,'Guest List'!D4:D157,B20)</f>
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A20,'Guest List'!D4:D182,B20)</f>
         <v/>
       </c>
     </row>
@@ -793,11 +793,11 @@
         </is>
       </c>
       <c r="C21" s="16">
-        <f>COUNTIFS('Guest List'!C4:C157,A21,'Guest List'!D4:D157,B21)</f>
+        <f>COUNTIFS('Guest List'!C4:C182,A21,'Guest List'!D4:D182,B21)</f>
         <v/>
       </c>
       <c r="D21" s="16">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A21,'Guest List'!D4:D157,B21)</f>
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A21,'Guest List'!D4:D182,B21)</f>
         <v/>
       </c>
     </row>
@@ -813,11 +813,11 @@
         </is>
       </c>
       <c r="C22" s="15">
-        <f>COUNTIFS('Guest List'!C4:C157,A22,'Guest List'!D4:D157,B22)</f>
+        <f>COUNTIFS('Guest List'!C4:C182,A22,'Guest List'!D4:D182,B22)</f>
         <v/>
       </c>
       <c r="D22" s="15">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A22,'Guest List'!D4:D157,B22)</f>
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A22,'Guest List'!D4:D182,B22)</f>
         <v/>
       </c>
     </row>
@@ -833,11 +833,11 @@
         </is>
       </c>
       <c r="C23" s="16">
-        <f>COUNTIFS('Guest List'!C4:C157,A23,'Guest List'!D4:D157,B23)</f>
+        <f>COUNTIFS('Guest List'!C4:C182,A23,'Guest List'!D4:D182,B23)</f>
         <v/>
       </c>
       <c r="D23" s="16">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A23,'Guest List'!D4:D157,B23)</f>
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A23,'Guest List'!D4:D182,B23)</f>
         <v/>
       </c>
     </row>
@@ -853,11 +853,11 @@
         </is>
       </c>
       <c r="C24" s="15">
-        <f>COUNTIFS('Guest List'!C4:C157,A24,'Guest List'!D4:D157,B24)</f>
+        <f>COUNTIFS('Guest List'!C4:C182,A24,'Guest List'!D4:D182,B24)</f>
         <v/>
       </c>
       <c r="D24" s="15">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A24,'Guest List'!D4:D157,B24)</f>
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A24,'Guest List'!D4:D182,B24)</f>
         <v/>
       </c>
     </row>
@@ -873,165 +873,185 @@
         </is>
       </c>
       <c r="C25" s="16">
-        <f>COUNTIFS('Guest List'!C4:C157,A25,'Guest List'!D4:D157,B25)</f>
+        <f>COUNTIFS('Guest List'!C4:C182,A25,'Guest List'!D4:D182,B25)</f>
         <v/>
       </c>
       <c r="D25" s="16">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A25,'Guest List'!D4:D157,B25)</f>
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A25,'Guest List'!D4:D182,B25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C26" s="15">
+        <f>COUNTIFS('Guest List'!C4:C182,A26,'Guest List'!D4:D182,B26)</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A26,'Guest List'!D4:D182,B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
           <t>Couple</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Bride &amp; Groom</t>
         </is>
       </c>
-      <c r="C26" s="15">
-        <f>COUNTIFS('Guest List'!C4:C157,A26,'Guest List'!D4:D157,B26)</f>
+      <c r="C27" s="16">
+        <f>COUNTIFS('Guest List'!C4:C182,A27,'Guest List'!D4:D182,B27)</f>
         <v/>
       </c>
-      <c r="D26" s="15">
-        <f>SUMIFS('Guest List'!F4:F157,'Guest List'!C4:C157,A26,'Guest List'!D4:D157,B26)</f>
+      <c r="D27" s="16">
+        <f>SUMIFS('Guest List'!F4:F182,'Guest List'!C4:C182,A27,'Guest List'!D4:D182,B27)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B27" s="17" t="n"/>
-      <c r="C27" s="17">
-        <f>SUM(C20:C26)</f>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17">
+        <f>SUM(C20:C27)</f>
         <v/>
       </c>
-      <c r="D27" s="17">
-        <f>SUM(D20:D26)</f>
+      <c r="D28" s="17">
+        <f>SUM(D20:D27)</f>
         <v/>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>BUDGET SNAPSHOT</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Estimated Total</t>
         </is>
       </c>
-      <c r="B30" s="10">
+      <c r="B31" s="10">
         <f>SUM(Budget!D4:D31)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Actual Total</t>
         </is>
       </c>
-      <c r="B31" s="18">
+      <c r="B32" s="18">
         <f>SUM(Budget!E4:E31)</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Paid to Date</t>
         </is>
       </c>
-      <c r="B32" s="10">
+      <c r="B33" s="10">
         <f>SUM(Budget!F4:F31)</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Balance Remaining</t>
         </is>
       </c>
-      <c r="B33" s="18">
+      <c r="B34" s="18">
         <f>SUM(Budget!G4:G31)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Budget Goal vs Estimate</t>
         </is>
       </c>
-      <c r="B34" s="10">
+      <c r="B35" s="10">
         <f>B7-SUM(Budget!D4:D31)</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>CHECKLIST PROGRESS</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Tasks - Done</t>
         </is>
       </c>
-      <c r="B37" s="13">
+      <c r="B38" s="13">
         <f>COUNTIF('Planning Checklist'!F4:F44,"Done")</f>
         <v/>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Tasks - In Progress</t>
         </is>
       </c>
-      <c r="B38" s="9">
+      <c r="B39" s="9">
         <f>COUNTIF('Planning Checklist'!F4:F44,"In Progress")</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Tasks - Not Started</t>
         </is>
       </c>
-      <c r="B39" s="13">
+      <c r="B40" s="13">
         <f>COUNTIF('Planning Checklist'!F4:F44,"Not Started")</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>% Complete</t>
         </is>
       </c>
-      <c r="B40" s="19">
+      <c r="B41" s="19">
         <f>IFERROR(COUNTIF('Planning Checklist'!F4:F44,"Done")/COUNTA('Planning Checklist'!A4:A44),0)</f>
         <v/>
       </c>
@@ -1039,12 +1059,12 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A30:D30"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1057,7 +1077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R158"/>
+  <dimension ref="A1:R183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9318,42 +9338,1406 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="5" t="n"/>
-      <c r="B158" s="25" t="inlineStr">
+      <c r="A158" s="16" t="n">
+        <v>155</v>
+      </c>
+      <c r="B158" s="23" t="inlineStr">
+        <is>
+          <t>Nathaniel</t>
+        </is>
+      </c>
+      <c r="C158" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D158" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E158" s="16" t="inlineStr">
+        <is>
+          <t>Nathaniel &amp; Rachel</t>
+        </is>
+      </c>
+      <c r="F158" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G158" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H158" s="16" t="n"/>
+      <c r="I158" s="16" t="n"/>
+      <c r="J158" s="16" t="n"/>
+      <c r="K158" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L158" s="16" t="n"/>
+      <c r="M158" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N158" s="16" t="n"/>
+      <c r="O158" s="16" t="n"/>
+      <c r="P158" s="16" t="n"/>
+      <c r="Q158" s="16" t="n"/>
+      <c r="R158" s="24" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="16" t="n">
+        <v>156</v>
+      </c>
+      <c r="B159" s="23" t="inlineStr">
+        <is>
+          <t>Rachel</t>
+        </is>
+      </c>
+      <c r="C159" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D159" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E159" s="16" t="inlineStr">
+        <is>
+          <t>Nathaniel &amp; Rachel</t>
+        </is>
+      </c>
+      <c r="F159" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G159" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H159" s="16" t="n"/>
+      <c r="I159" s="16" t="n"/>
+      <c r="J159" s="16" t="n"/>
+      <c r="K159" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L159" s="16" t="n"/>
+      <c r="M159" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N159" s="16" t="n"/>
+      <c r="O159" s="16" t="n"/>
+      <c r="P159" s="16" t="n"/>
+      <c r="Q159" s="16" t="n"/>
+      <c r="R159" s="24" t="inlineStr">
+        <is>
+          <t>Last name to confirm - not Rachel Lane or Rachel Guy</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="15" t="n">
+        <v>157</v>
+      </c>
+      <c r="B160" s="21" t="inlineStr">
+        <is>
+          <t>Viet</t>
+        </is>
+      </c>
+      <c r="C160" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D160" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E160" s="15" t="inlineStr">
+        <is>
+          <t>Viet &amp; Debbie</t>
+        </is>
+      </c>
+      <c r="F160" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G160" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H160" s="15" t="n"/>
+      <c r="I160" s="15" t="n"/>
+      <c r="J160" s="15" t="n"/>
+      <c r="K160" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L160" s="15" t="n"/>
+      <c r="M160" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N160" s="15" t="n"/>
+      <c r="O160" s="15" t="n"/>
+      <c r="P160" s="15" t="n"/>
+      <c r="Q160" s="15" t="n"/>
+      <c r="R160" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="15" t="n">
+        <v>158</v>
+      </c>
+      <c r="B161" s="21" t="inlineStr">
+        <is>
+          <t>Debbie</t>
+        </is>
+      </c>
+      <c r="C161" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D161" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E161" s="15" t="inlineStr">
+        <is>
+          <t>Viet &amp; Debbie</t>
+        </is>
+      </c>
+      <c r="F161" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G161" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H161" s="15" t="n"/>
+      <c r="I161" s="15" t="n"/>
+      <c r="J161" s="15" t="n"/>
+      <c r="K161" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L161" s="15" t="n"/>
+      <c r="M161" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N161" s="15" t="n"/>
+      <c r="O161" s="15" t="n"/>
+      <c r="P161" s="15" t="n"/>
+      <c r="Q161" s="15" t="n"/>
+      <c r="R161" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="16" t="n">
+        <v>159</v>
+      </c>
+      <c r="B162" s="23" t="inlineStr">
+        <is>
+          <t>Noah</t>
+        </is>
+      </c>
+      <c r="C162" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D162" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E162" s="16" t="inlineStr">
+        <is>
+          <t>Noah &amp; Emily</t>
+        </is>
+      </c>
+      <c r="F162" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G162" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H162" s="16" t="n"/>
+      <c r="I162" s="16" t="n"/>
+      <c r="J162" s="16" t="n"/>
+      <c r="K162" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L162" s="16" t="n"/>
+      <c r="M162" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N162" s="16" t="n"/>
+      <c r="O162" s="16" t="n"/>
+      <c r="P162" s="16" t="n"/>
+      <c r="Q162" s="16" t="n"/>
+      <c r="R162" s="24" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="16" t="n">
+        <v>160</v>
+      </c>
+      <c r="B163" s="23" t="inlineStr">
+        <is>
+          <t>Emily</t>
+        </is>
+      </c>
+      <c r="C163" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D163" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E163" s="16" t="inlineStr">
+        <is>
+          <t>Noah &amp; Emily</t>
+        </is>
+      </c>
+      <c r="F163" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G163" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H163" s="16" t="n"/>
+      <c r="I163" s="16" t="n"/>
+      <c r="J163" s="16" t="n"/>
+      <c r="K163" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L163" s="16" t="n"/>
+      <c r="M163" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N163" s="16" t="n"/>
+      <c r="O163" s="16" t="n"/>
+      <c r="P163" s="16" t="n"/>
+      <c r="Q163" s="16" t="n"/>
+      <c r="R163" s="24" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="15" t="n">
+        <v>161</v>
+      </c>
+      <c r="B164" s="21" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="C164" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D164" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E164" s="15" t="inlineStr">
+        <is>
+          <t>Michael &amp; Alisa</t>
+        </is>
+      </c>
+      <c r="F164" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G164" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H164" s="15" t="n"/>
+      <c r="I164" s="15" t="n"/>
+      <c r="J164" s="15" t="n"/>
+      <c r="K164" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L164" s="15" t="n"/>
+      <c r="M164" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N164" s="15" t="n"/>
+      <c r="O164" s="15" t="n"/>
+      <c r="P164" s="15" t="n"/>
+      <c r="Q164" s="15" t="n"/>
+      <c r="R164" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm - not Michael Rumende or Michael on row 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="15" t="n">
+        <v>162</v>
+      </c>
+      <c r="B165" s="21" t="inlineStr">
+        <is>
+          <t>Alisa</t>
+        </is>
+      </c>
+      <c r="C165" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D165" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E165" s="15" t="inlineStr">
+        <is>
+          <t>Michael &amp; Alisa</t>
+        </is>
+      </c>
+      <c r="F165" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G165" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H165" s="15" t="n"/>
+      <c r="I165" s="15" t="n"/>
+      <c r="J165" s="15" t="n"/>
+      <c r="K165" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L165" s="15" t="n"/>
+      <c r="M165" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N165" s="15" t="n"/>
+      <c r="O165" s="15" t="n"/>
+      <c r="P165" s="15" t="n"/>
+      <c r="Q165" s="15" t="n"/>
+      <c r="R165" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="16" t="n">
+        <v>163</v>
+      </c>
+      <c r="B166" s="23" t="inlineStr">
+        <is>
+          <t>Grant</t>
+        </is>
+      </c>
+      <c r="C166" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D166" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E166" s="16" t="inlineStr">
+        <is>
+          <t>Grant &amp; Samantha</t>
+        </is>
+      </c>
+      <c r="F166" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G166" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H166" s="16" t="n"/>
+      <c r="I166" s="16" t="n"/>
+      <c r="J166" s="16" t="n"/>
+      <c r="K166" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L166" s="16" t="n"/>
+      <c r="M166" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N166" s="16" t="n"/>
+      <c r="O166" s="16" t="n"/>
+      <c r="P166" s="16" t="n"/>
+      <c r="Q166" s="16" t="n"/>
+      <c r="R166" s="24" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="n">
+        <v>164</v>
+      </c>
+      <c r="B167" s="23" t="inlineStr">
+        <is>
+          <t>Samantha</t>
+        </is>
+      </c>
+      <c r="C167" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D167" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E167" s="16" t="inlineStr">
+        <is>
+          <t>Grant &amp; Samantha</t>
+        </is>
+      </c>
+      <c r="F167" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G167" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H167" s="16" t="n"/>
+      <c r="I167" s="16" t="n"/>
+      <c r="J167" s="16" t="n"/>
+      <c r="K167" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L167" s="16" t="n"/>
+      <c r="M167" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N167" s="16" t="n"/>
+      <c r="O167" s="16" t="n"/>
+      <c r="P167" s="16" t="n"/>
+      <c r="Q167" s="16" t="n"/>
+      <c r="R167" s="24" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="15" t="n">
+        <v>165</v>
+      </c>
+      <c r="B168" s="21" t="inlineStr">
+        <is>
+          <t>Garrett</t>
+        </is>
+      </c>
+      <c r="C168" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D168" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E168" s="15" t="inlineStr">
+        <is>
+          <t>Garrett &amp; Moriah</t>
+        </is>
+      </c>
+      <c r="F168" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G168" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H168" s="15" t="n"/>
+      <c r="I168" s="15" t="n"/>
+      <c r="J168" s="15" t="n"/>
+      <c r="K168" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L168" s="15" t="n"/>
+      <c r="M168" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N168" s="15" t="n"/>
+      <c r="O168" s="15" t="n"/>
+      <c r="P168" s="15" t="n"/>
+      <c r="Q168" s="15" t="n"/>
+      <c r="R168" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm - not Garrett Thurmond</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="15" t="n">
+        <v>166</v>
+      </c>
+      <c r="B169" s="21" t="inlineStr">
+        <is>
+          <t>Moriah</t>
+        </is>
+      </c>
+      <c r="C169" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D169" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E169" s="15" t="inlineStr">
+        <is>
+          <t>Garrett &amp; Moriah</t>
+        </is>
+      </c>
+      <c r="F169" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G169" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H169" s="15" t="n"/>
+      <c r="I169" s="15" t="n"/>
+      <c r="J169" s="15" t="n"/>
+      <c r="K169" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L169" s="15" t="n"/>
+      <c r="M169" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N169" s="15" t="n"/>
+      <c r="O169" s="15" t="n"/>
+      <c r="P169" s="15" t="n"/>
+      <c r="Q169" s="15" t="n"/>
+      <c r="R169" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="16" t="n">
+        <v>167</v>
+      </c>
+      <c r="B170" s="23" t="inlineStr">
+        <is>
+          <t>Madeleine Harris</t>
+        </is>
+      </c>
+      <c r="C170" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D170" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E170" s="16" t="inlineStr">
+        <is>
+          <t>Harris</t>
+        </is>
+      </c>
+      <c r="F170" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G170" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H170" s="16" t="n"/>
+      <c r="I170" s="16" t="n"/>
+      <c r="J170" s="16" t="n"/>
+      <c r="K170" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L170" s="16" t="n"/>
+      <c r="M170" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N170" s="16" t="n"/>
+      <c r="O170" s="16" t="n"/>
+      <c r="P170" s="16" t="n"/>
+      <c r="Q170" s="16" t="n"/>
+      <c r="R170" s="24" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="15" t="n">
+        <v>168</v>
+      </c>
+      <c r="B171" s="21" t="inlineStr">
+        <is>
+          <t>Bee Icayan</t>
+        </is>
+      </c>
+      <c r="C171" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D171" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E171" s="15" t="inlineStr">
+        <is>
+          <t>Icayan</t>
+        </is>
+      </c>
+      <c r="F171" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G171" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H171" s="15" t="n"/>
+      <c r="I171" s="15" t="n"/>
+      <c r="J171" s="15" t="n"/>
+      <c r="K171" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L171" s="15" t="n"/>
+      <c r="M171" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N171" s="15" t="n"/>
+      <c r="O171" s="15" t="n"/>
+      <c r="P171" s="15" t="n"/>
+      <c r="Q171" s="15" t="n"/>
+      <c r="R171" s="22" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="16" t="n">
+        <v>169</v>
+      </c>
+      <c r="B172" s="23" t="inlineStr">
+        <is>
+          <t>Anna Ruth Flagg</t>
+        </is>
+      </c>
+      <c r="C172" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D172" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E172" s="16" t="inlineStr">
+        <is>
+          <t>Flagg</t>
+        </is>
+      </c>
+      <c r="F172" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G172" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H172" s="16" t="n"/>
+      <c r="I172" s="16" t="n"/>
+      <c r="J172" s="16" t="n"/>
+      <c r="K172" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L172" s="16" t="n"/>
+      <c r="M172" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N172" s="16" t="n"/>
+      <c r="O172" s="16" t="n"/>
+      <c r="P172" s="16" t="n"/>
+      <c r="Q172" s="16" t="n"/>
+      <c r="R172" s="24" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="15" t="n">
+        <v>170</v>
+      </c>
+      <c r="B173" s="21" t="inlineStr">
+        <is>
+          <t>Rhiannon Beard</t>
+        </is>
+      </c>
+      <c r="C173" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D173" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E173" s="15" t="inlineStr">
+        <is>
+          <t>Beard</t>
+        </is>
+      </c>
+      <c r="F173" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G173" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H173" s="15" t="n"/>
+      <c r="I173" s="15" t="n"/>
+      <c r="J173" s="15" t="n"/>
+      <c r="K173" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L173" s="15" t="n"/>
+      <c r="M173" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N173" s="15" t="n"/>
+      <c r="O173" s="15" t="n"/>
+      <c r="P173" s="15" t="n"/>
+      <c r="Q173" s="15" t="n"/>
+      <c r="R173" s="22" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="15" t="n">
+        <v>171</v>
+      </c>
+      <c r="B174" s="21" t="inlineStr">
+        <is>
+          <t>Rhiannon Beard's +1</t>
+        </is>
+      </c>
+      <c r="C174" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D174" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E174" s="15" t="inlineStr">
+        <is>
+          <t>Beard</t>
+        </is>
+      </c>
+      <c r="F174" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G174" s="15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H174" s="15" t="n"/>
+      <c r="I174" s="15" t="n"/>
+      <c r="J174" s="15" t="n"/>
+      <c r="K174" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L174" s="15" t="n"/>
+      <c r="M174" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N174" s="15" t="n"/>
+      <c r="O174" s="15" t="n"/>
+      <c r="P174" s="15" t="n"/>
+      <c r="Q174" s="15" t="n"/>
+      <c r="R174" s="22" t="inlineStr">
+        <is>
+          <t>+1 to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="16" t="n">
+        <v>172</v>
+      </c>
+      <c r="B175" s="23" t="inlineStr">
+        <is>
+          <t>Megan Rogers</t>
+        </is>
+      </c>
+      <c r="C175" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D175" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E175" s="16" t="inlineStr">
+        <is>
+          <t>Rogers</t>
+        </is>
+      </c>
+      <c r="F175" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G175" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H175" s="16" t="n"/>
+      <c r="I175" s="16" t="n"/>
+      <c r="J175" s="16" t="n"/>
+      <c r="K175" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L175" s="16" t="n"/>
+      <c r="M175" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N175" s="16" t="n"/>
+      <c r="O175" s="16" t="n"/>
+      <c r="P175" s="16" t="n"/>
+      <c r="Q175" s="16" t="n"/>
+      <c r="R175" s="24" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="15" t="n">
+        <v>173</v>
+      </c>
+      <c r="B176" s="21" t="inlineStr">
+        <is>
+          <t>Norma Street</t>
+        </is>
+      </c>
+      <c r="C176" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D176" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E176" s="15" t="inlineStr">
+        <is>
+          <t>Street</t>
+        </is>
+      </c>
+      <c r="F176" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G176" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H176" s="15" t="n"/>
+      <c r="I176" s="15" t="n"/>
+      <c r="J176" s="15" t="n"/>
+      <c r="K176" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L176" s="15" t="n"/>
+      <c r="M176" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N176" s="15" t="n"/>
+      <c r="O176" s="15" t="n"/>
+      <c r="P176" s="15" t="n"/>
+      <c r="Q176" s="15" t="n"/>
+      <c r="R176" s="22" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="15" t="n">
+        <v>174</v>
+      </c>
+      <c r="B177" s="21" t="inlineStr">
+        <is>
+          <t>Jay Street</t>
+        </is>
+      </c>
+      <c r="C177" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D177" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E177" s="15" t="inlineStr">
+        <is>
+          <t>Street</t>
+        </is>
+      </c>
+      <c r="F177" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G177" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H177" s="15" t="n"/>
+      <c r="I177" s="15" t="n"/>
+      <c r="J177" s="15" t="n"/>
+      <c r="K177" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L177" s="15" t="n"/>
+      <c r="M177" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N177" s="15" t="n"/>
+      <c r="O177" s="15" t="n"/>
+      <c r="P177" s="15" t="n"/>
+      <c r="Q177" s="15" t="n"/>
+      <c r="R177" s="22" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="16" t="n">
+        <v>175</v>
+      </c>
+      <c r="B178" s="23" t="inlineStr">
+        <is>
+          <t>Jackie Santander</t>
+        </is>
+      </c>
+      <c r="C178" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D178" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E178" s="16" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="F178" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G178" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H178" s="16" t="n"/>
+      <c r="I178" s="16" t="n"/>
+      <c r="J178" s="16" t="n"/>
+      <c r="K178" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L178" s="16" t="n"/>
+      <c r="M178" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N178" s="16" t="n"/>
+      <c r="O178" s="16" t="n"/>
+      <c r="P178" s="16" t="n"/>
+      <c r="Q178" s="16" t="n"/>
+      <c r="R178" s="24" t="inlineStr">
+        <is>
+          <t>Possible overlap with Jackie on row 91 - check</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="16" t="n">
+        <v>176</v>
+      </c>
+      <c r="B179" s="23" t="inlineStr">
+        <is>
+          <t>Chris Santander</t>
+        </is>
+      </c>
+      <c r="C179" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D179" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E179" s="16" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="F179" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G179" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H179" s="16" t="n"/>
+      <c r="I179" s="16" t="n"/>
+      <c r="J179" s="16" t="n"/>
+      <c r="K179" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L179" s="16" t="n"/>
+      <c r="M179" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N179" s="16" t="n"/>
+      <c r="O179" s="16" t="n"/>
+      <c r="P179" s="16" t="n"/>
+      <c r="Q179" s="16" t="n"/>
+      <c r="R179" s="24" t="inlineStr">
+        <is>
+          <t>Possible overlap with Chris / Chris' wife on rows 101-102 - check</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="15" t="n">
+        <v>177</v>
+      </c>
+      <c r="B180" s="21" t="inlineStr">
+        <is>
+          <t>Sheona</t>
+        </is>
+      </c>
+      <c r="C180" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D180" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E180" s="15" t="inlineStr">
+        <is>
+          <t>Sheona &amp; Issac</t>
+        </is>
+      </c>
+      <c r="F180" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G180" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H180" s="15" t="n"/>
+      <c r="I180" s="15" t="n"/>
+      <c r="J180" s="15" t="n"/>
+      <c r="K180" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L180" s="15" t="n"/>
+      <c r="M180" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N180" s="15" t="n"/>
+      <c r="O180" s="15" t="n"/>
+      <c r="P180" s="15" t="n"/>
+      <c r="Q180" s="15" t="n"/>
+      <c r="R180" s="22" t="inlineStr">
+        <is>
+          <t>Last name to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="15" t="n">
+        <v>178</v>
+      </c>
+      <c r="B181" s="21" t="inlineStr">
+        <is>
+          <t>Issac</t>
+        </is>
+      </c>
+      <c r="C181" s="15" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D181" s="15" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E181" s="15" t="inlineStr">
+        <is>
+          <t>Sheona &amp; Issac</t>
+        </is>
+      </c>
+      <c r="F181" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G181" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H181" s="15" t="n"/>
+      <c r="I181" s="15" t="n"/>
+      <c r="J181" s="15" t="n"/>
+      <c r="K181" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L181" s="15" t="n"/>
+      <c r="M181" s="15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N181" s="15" t="n"/>
+      <c r="O181" s="15" t="n"/>
+      <c r="P181" s="15" t="n"/>
+      <c r="Q181" s="15" t="n"/>
+      <c r="R181" s="22" t="inlineStr">
+        <is>
+          <t>Spelling to confirm - Issac or Isaac?</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="16" t="n">
+        <v>179</v>
+      </c>
+      <c r="B182" s="23" t="inlineStr">
+        <is>
+          <t>Rachel Guy</t>
+        </is>
+      </c>
+      <c r="C182" s="16" t="inlineStr">
+        <is>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="D182" s="16" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="E182" s="16" t="inlineStr">
+        <is>
+          <t>Guy</t>
+        </is>
+      </c>
+      <c r="F182" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G182" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H182" s="16" t="n"/>
+      <c r="I182" s="16" t="n"/>
+      <c r="J182" s="16" t="n"/>
+      <c r="K182" s="16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L182" s="16" t="n"/>
+      <c r="M182" s="16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="N182" s="16" t="n"/>
+      <c r="O182" s="16" t="n"/>
+      <c r="P182" s="16" t="n"/>
+      <c r="Q182" s="16" t="n"/>
+      <c r="R182" s="24" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="n"/>
+      <c r="B183" s="25" t="inlineStr">
         <is>
           <t>TOTALS</t>
         </is>
       </c>
-      <c r="C158" s="5" t="n"/>
-      <c r="D158" s="5" t="n"/>
-      <c r="E158" s="5" t="n"/>
-      <c r="F158" s="25">
-        <f>SUM(F4:F157)</f>
+      <c r="C183" s="5" t="n"/>
+      <c r="D183" s="5" t="n"/>
+      <c r="E183" s="5" t="n"/>
+      <c r="F183" s="25">
+        <f>SUM(F4:F182)</f>
         <v/>
       </c>
-      <c r="G158" s="5" t="n"/>
-      <c r="H158" s="5" t="n"/>
-      <c r="I158" s="5" t="n"/>
-      <c r="J158" s="5" t="n"/>
-      <c r="K158" s="5" t="n"/>
-      <c r="L158" s="5" t="n"/>
-      <c r="M158" s="5" t="n"/>
-      <c r="N158" s="25">
-        <f>SUM(N4:N157)</f>
+      <c r="G183" s="5" t="n"/>
+      <c r="H183" s="5" t="n"/>
+      <c r="I183" s="5" t="n"/>
+      <c r="J183" s="5" t="n"/>
+      <c r="K183" s="5" t="n"/>
+      <c r="L183" s="5" t="n"/>
+      <c r="M183" s="5" t="n"/>
+      <c r="N183" s="25">
+        <f>SUM(N4:N182)</f>
         <v/>
       </c>
-      <c r="O158" s="5" t="n"/>
-      <c r="P158" s="5" t="n"/>
-      <c r="Q158" s="5" t="n"/>
-      <c r="R158" s="5" t="n"/>
+      <c r="O183" s="5" t="n"/>
+      <c r="P183" s="5" t="n"/>
+      <c r="Q183" s="5" t="n"/>
+      <c r="R183" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:R157"/>
+  <autoFilter ref="A3:R182"/>
   <mergeCells count="2">
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="A1:R1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M4:M157">
+  <conditionalFormatting sqref="M4:M182">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
@@ -9362,10 +10746,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G4:G157 K4:L157 P4:Q157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4:G182 K4:L182 P4:Q182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,TBD"</formula1>
     </dataValidation>
-    <dataValidation sqref="M4:M157" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M4:M182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>